<commit_message>
style: center Excel export cells and add table borders
</commit_message>
<xml_diff>
--- a/backend/assets/export-template.xlsx
+++ b/backend/assets/export-template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Приоритеты" sheetId="1" r:id="R9125be77dedf4f7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все счета" sheetId="2" r:id="R8fe990b7e6b64191"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сообщества" sheetId="3" r:id="R2afaabbbbfab49ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="О выгрузке" sheetId="4" r:id="Rcacae20989b54531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Приоритеты" sheetId="1" r:id="Rf15b9cb135184b4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все счета" sheetId="2" r:id="R20ff98c061dd4683"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сообщества" sheetId="3" r:id="R112f22c7d3fd4c17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="О выгрузке" sheetId="4" r:id="R73cfbf80b20a43d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,13 +52,27 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF8497A3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF8497A3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF8497A3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8497A3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -75,9 +89,54 @@
     <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -289,36 +348,36 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="18" t="str">
         <x:v>rank</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="18" t="str">
         <x:v>gid</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="18" t="str">
         <x:v>role</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="18" t="str">
         <x:v>priority_score</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" s="18" t="str">
         <x:v>why</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="5" t="n">
+      <x:c r="A2" s="19" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="str">
+      <x:c r="B2" s="20" t="str">
         <x:v>100000000000000001</x:v>
       </x:c>
-      <x:c r="C2" s="7" t="str">
+      <x:c r="C2" s="20" t="str">
         <x:v>transit</x:v>
       </x:c>
-      <x:c r="D2" s="9" t="n">
+      <x:c r="D2" s="21" t="n">
         <x:v>0.123456</x:v>
       </x:c>
-      <x:c r="E2" s="7" t="str">
+      <x:c r="E2" s="20" t="str">
         <x:v>Объяснение приоритета</x:v>
       </x:c>
     </x:row>
@@ -340,42 +399,42 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="18" t="str">
         <x:v>gid</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="18" t="str">
         <x:v>role</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="18" t="str">
         <x:v>role_score</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="18" t="str">
         <x:v>cluster_id</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" s="18" t="str">
         <x:v>priority_score</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="str">
+      <x:c r="F1" s="18" t="str">
         <x:v>evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="7" t="str">
+      <x:c r="A2" s="20" t="str">
         <x:v>100000000000000001</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="str">
+      <x:c r="B2" s="20" t="str">
         <x:v>transit</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="n">
+      <x:c r="C2" s="21" t="n">
         <x:v>0.123456</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="n">
+      <x:c r="D2" s="19" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E2" s="9" t="n">
+      <x:c r="E2" s="21" t="n">
         <x:v>0.123456</x:v>
       </x:c>
-      <x:c r="F2" s="7" t="str">
+      <x:c r="F2" s="20" t="str">
         <x:v>Подтверждающие факты</x:v>
       </x:c>
     </x:row>
@@ -397,42 +456,42 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="18" t="str">
         <x:v>cluster_id</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="18" t="str">
         <x:v>n_nodes</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="18" t="str">
         <x:v>n_seed</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="18" t="str">
         <x:v>sum_kzt_internal</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" s="18" t="str">
         <x:v>top_gids</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="str">
+      <x:c r="F1" s="18" t="str">
         <x:v>hypothesis</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="5" t="n">
+      <x:c r="A2" s="19" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="n">
+      <x:c r="B2" s="19" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="n">
+      <x:c r="C2" s="19" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="n">
+      <x:c r="D2" s="26" t="n">
         <x:v>1234.56</x:v>
       </x:c>
-      <x:c r="E2" s="7" t="str">
+      <x:c r="E2" s="20" t="str">
         <x:v>100000000000000001</x:v>
       </x:c>
-      <x:c r="F2" s="7" t="str">
+      <x:c r="F2" s="20" t="str">
         <x:v>Гипотеза сообщества</x:v>
       </x:c>
     </x:row>
@@ -450,18 +509,18 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="18" t="str">
         <x:v>Параметр</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="18" t="str">
         <x:v>Значение</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="7" t="str">
+      <x:c r="A2" s="20" t="str">
         <x:v>Версия метода</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="str">
+      <x:c r="B2" s="20" t="str">
         <x:v>1.1.0</x:v>
       </x:c>
     </x:row>

</xml_diff>